<commit_message>
Publish ACC page: remove draft status, wording corrections, mobile fix
</commit_message>
<xml_diff>
--- a/data/acc/ACC Aggregate Results 2019 and 2026.xlsx
+++ b/data/acc/ACC Aggregate Results 2019 and 2026.xlsx
@@ -1308,7 +1308,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>No entry-level data, titles or names are included. Languages with fewer than 5 titles are grouped; topic-share bins with fewer than 20 titles are omitted.</t>
+          <t>No entry-level data, titles or names are included. Languages with fewer than 5 titles in both editions are grouped; topic-share bins with fewer than 20 titles are omitted.</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2. Every 2019 entry and every new 2026 entry was checked against its parsed fields with AI assistance; every disagreement was resolved by hand. Repeated 2026 entries inherited their 2019 checks (random audit: 0 errors in 80).</t>
+          <t>2. Every 2019 entry and every new 2026 entry was checked against its parsed fields with AI assistance (Claude). Every 2019 disagreement was ruled on by hand; in 2026 the same rulings were applied and the cases they did not settle were decided by hand. Repeated 2026 entries inherited their 2019 checks (random audit: no substantive errors in 80).</t>
         </is>
       </c>
     </row>

</xml_diff>